<commit_message>
made forecast work with mock data
</commit_message>
<xml_diff>
--- a/packages/backend/files/Produktionszeit_Warenfluss_Hackathon_Teilnehmer.xlsx
+++ b/packages/backend/files/Produktionszeit_Warenfluss_Hackathon_Teilnehmer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ap8c3/IdeaProjects/Hackathon/eleo-mind/packages/backend/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AF19A45-AC21-1345-B96D-95C0A4C05752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13D3DB1-55DE-B34A-B882-2ABBE7A9C9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="17380" xr2:uid="{89DEC141-2149-4C1E-98A2-7345C7C4F172}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="17380" activeTab="4" xr2:uid="{89DEC141-2149-4C1E-98A2-7345C7C4F172}"/>
   </bookViews>
   <sheets>
     <sheet name="Produktsparte 1_Produktionszeit" sheetId="8" r:id="rId1"/>
@@ -23,9 +23,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Produktsparte 1_Produktionszeit'!$A$1:$J$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produktsparte 1_Warenfluss'!$A$1:$J$45</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Produktsparte 2_Produktionzeit'!$A$1:$J$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Produktsparte 2_Produktionzeit'!$A$1:$J$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Produktsparte 2_Warenfluss'!$A$1:$J$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Produktsparte 3_Produktionszeit'!$A$1:$I$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Produktsparte 3_Produktionszeit'!$A$1:$I$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Produktsparte 3_Warenfluss'!$A$1:$I$75</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="888" uniqueCount="218">
   <si>
     <t>SKU</t>
   </si>
@@ -700,6 +700,9 @@
   </si>
   <si>
     <t>SZ2103sf</t>
+  </si>
+  <si>
+    <t>920302, 920304, 920306, 920308</t>
   </si>
 </sst>
 </file>
@@ -2754,7 +2757,7 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="11" t="s">
-        <v>62</v>
+        <v>217</v>
       </c>
       <c r="B50" s="11" t="s">
         <v>59</v>
@@ -7218,7 +7221,7 @@
   <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="3" width="13.5" bestFit="1" customWidth="1"/>
@@ -7740,25 +7743,25 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C17" s="5">
         <v>0</v>
       </c>
       <c r="D17" s="5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E17" s="5">
         <v>0</v>
       </c>
-      <c r="F17" s="9">
-        <v>60</v>
+      <c r="F17" s="5">
+        <v>0</v>
       </c>
       <c r="G17" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H17" s="9">
         <v>0</v>
@@ -7772,10 +7775,10 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C18" s="5">
         <v>0</v>
@@ -7793,7 +7796,7 @@
         <v>0</v>
       </c>
       <c r="H18" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I18" s="9">
         <v>0</v>
@@ -7804,10 +7807,10 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="10" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C19" s="5">
         <v>0</v>
@@ -7822,10 +7825,10 @@
         <v>0</v>
       </c>
       <c r="G19" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H19" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I19" s="9">
         <v>0</v>
@@ -7836,10 +7839,10 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C20" s="5">
         <v>0</v>
@@ -7868,10 +7871,10 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C21" s="5">
         <v>0</v>
@@ -7886,7 +7889,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H21" s="9">
         <v>0</v>
@@ -7900,10 +7903,10 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="10" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C22" s="5">
         <v>0</v>
@@ -7921,7 +7924,7 @@
         <v>0</v>
       </c>
       <c r="H22" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I22" s="9">
         <v>0</v>
@@ -7932,10 +7935,10 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C23" s="5">
         <v>0</v>
@@ -7950,10 +7953,10 @@
         <v>0</v>
       </c>
       <c r="G23" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H23" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I23" s="9">
         <v>0</v>
@@ -7964,10 +7967,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C24" s="5">
         <v>0</v>
@@ -7996,25 +7999,25 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C25" s="5">
         <v>0</v>
       </c>
       <c r="D25" s="5">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E25" s="5">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F25" s="5">
         <v>0</v>
       </c>
       <c r="G25" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H25" s="9">
         <v>0</v>
@@ -8028,10 +8031,10 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C26" s="5">
         <v>0</v>
@@ -8049,7 +8052,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I26" s="9">
         <v>0</v>
@@ -8060,10 +8063,10 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C27" s="5">
         <v>0</v>
@@ -8078,10 +8081,10 @@
         <v>0</v>
       </c>
       <c r="G27" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H27" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I27" s="9">
         <v>0</v>
@@ -8092,10 +8095,10 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C28" s="5">
         <v>0</v>
@@ -8124,25 +8127,25 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C29" s="5">
         <v>0</v>
       </c>
       <c r="D29" s="5">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E29" s="5">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F29" s="5">
         <v>0</v>
       </c>
       <c r="G29" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H29" s="9">
         <v>0</v>
@@ -8156,10 +8159,10 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C30" s="5">
         <v>0</v>
@@ -8177,7 +8180,7 @@
         <v>0</v>
       </c>
       <c r="H30" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I30" s="9">
         <v>0</v>
@@ -8188,10 +8191,10 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C31" s="5">
         <v>0</v>
@@ -8206,10 +8209,10 @@
         <v>0</v>
       </c>
       <c r="G31" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H31" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I31" s="9">
         <v>0</v>
@@ -8220,10 +8223,10 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C32" s="5">
         <v>0</v>
@@ -8252,10 +8255,10 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C33" s="5">
         <v>0</v>
@@ -8270,7 +8273,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H33" s="9">
         <v>0</v>
@@ -8284,10 +8287,10 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C34" s="5">
         <v>0</v>
@@ -8305,7 +8308,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I34" s="9">
         <v>0</v>
@@ -8316,10 +8319,10 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C35" s="5">
         <v>0</v>
@@ -8334,10 +8337,10 @@
         <v>0</v>
       </c>
       <c r="G35" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H35" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I35" s="9">
         <v>0</v>
@@ -8348,10 +8351,10 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C36" s="5">
         <v>0</v>
@@ -8380,10 +8383,10 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C37" s="5">
         <v>0</v>
@@ -8398,7 +8401,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H37" s="9">
         <v>0</v>
@@ -8412,10 +8415,10 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C38" s="5">
         <v>0</v>
@@ -8433,7 +8436,7 @@
         <v>0</v>
       </c>
       <c r="H38" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I38" s="9">
         <v>0</v>
@@ -8444,10 +8447,10 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C39" s="5">
         <v>0</v>
@@ -8462,10 +8465,10 @@
         <v>0</v>
       </c>
       <c r="G39" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H39" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I39" s="9">
         <v>0</v>
@@ -8476,10 +8479,10 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C40" s="5">
         <v>0</v>
@@ -8508,25 +8511,25 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C41" s="5">
         <v>0</v>
       </c>
       <c r="D41" s="5">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="E41" s="5">
         <v>0</v>
       </c>
       <c r="F41" s="5">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="G41" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H41" s="9">
         <v>0</v>
@@ -8540,10 +8543,10 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C42" s="5">
         <v>0</v>
@@ -8561,7 +8564,7 @@
         <v>0</v>
       </c>
       <c r="H42" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I42" s="9">
         <v>0</v>
@@ -8572,10 +8575,10 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C43" s="5">
         <v>0</v>
@@ -8590,10 +8593,10 @@
         <v>60</v>
       </c>
       <c r="G43" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H43" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I43" s="9">
         <v>0</v>
@@ -8604,10 +8607,10 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C44" s="5">
         <v>0</v>
@@ -8636,10 +8639,10 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="10" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>59</v>
+        <v>11</v>
       </c>
       <c r="C45" s="5">
         <v>0</v>
@@ -8654,7 +8657,7 @@
         <v>60</v>
       </c>
       <c r="G45" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H45" s="9">
         <v>0</v>
@@ -8668,10 +8671,10 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C46" s="5">
         <v>0</v>
@@ -8689,7 +8692,7 @@
         <v>0</v>
       </c>
       <c r="H46" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I46" s="9">
         <v>0</v>
@@ -8700,10 +8703,10 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="10" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C47" s="5">
         <v>0</v>
@@ -8718,10 +8721,10 @@
         <v>60</v>
       </c>
       <c r="G47" s="9">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H47" s="9">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I47" s="9">
         <v>0</v>
@@ -8732,10 +8735,10 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="C48" s="5">
         <v>0</v>
@@ -8762,40 +8765,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B49" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C49" s="5">
-        <v>0</v>
-      </c>
-      <c r="D49" s="5">
-        <v>0</v>
-      </c>
-      <c r="E49" s="5">
-        <v>0</v>
-      </c>
-      <c r="F49" s="5">
-        <v>60</v>
-      </c>
-      <c r="G49" s="9">
-        <v>15</v>
-      </c>
-      <c r="H49" s="9">
-        <v>0</v>
-      </c>
-      <c r="I49" s="9">
-        <v>0</v>
-      </c>
-      <c r="J49" s="9">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:J49" xr:uid="{DFD78E8A-34F1-4E1A-BE10-09763EA23C2F}"/>
+  <autoFilter ref="A1:J48" xr:uid="{DFD78E8A-34F1-4E1A-BE10-09763EA23C2F}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10357,10 +10328,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B237460F-1A26-43E8-9FBD-2B515F45BBA9}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:J75"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -10406,7 +10377,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>146</v>
       </c>
@@ -10438,7 +10409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>147</v>
       </c>
@@ -10470,7 +10441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>148</v>
       </c>
@@ -10502,7 +10473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>149</v>
       </c>
@@ -10534,7 +10505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>150</v>
       </c>
@@ -10566,7 +10537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>151</v>
       </c>
@@ -10598,7 +10569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>152</v>
       </c>
@@ -10630,685 +10601,685 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B9" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="5">
+        <v>15</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5">
+        <v>0</v>
+      </c>
+      <c r="I9" s="5">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="5">
+        <v>15</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0</v>
+      </c>
+      <c r="F10" s="5">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5">
+        <v>15</v>
+      </c>
+      <c r="I10" s="5">
+        <v>0</v>
+      </c>
+      <c r="J10" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="5">
+        <v>15</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0</v>
+      </c>
+      <c r="F11" s="5">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5">
+        <v>15</v>
+      </c>
+      <c r="H11" s="5">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="5">
-        <v>15</v>
-      </c>
-      <c r="D9" s="5">
-        <v>0</v>
-      </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="5">
-        <v>15</v>
-      </c>
-      <c r="H9" s="5">
-        <v>0</v>
-      </c>
-      <c r="I9" s="5">
-        <v>0</v>
-      </c>
-      <c r="J9" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="B10" s="10" t="s">
+      <c r="C12" s="5">
+        <v>15</v>
+      </c>
+      <c r="D12" s="5">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5">
+        <v>0</v>
+      </c>
+      <c r="F12" s="5">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5">
+        <v>15</v>
+      </c>
+      <c r="H12" s="5">
+        <v>0</v>
+      </c>
+      <c r="I12" s="5">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="5">
-        <v>15</v>
-      </c>
-      <c r="D10" s="5">
-        <v>0</v>
-      </c>
-      <c r="E10" s="5">
-        <v>0</v>
-      </c>
-      <c r="F10" s="5">
-        <v>0</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="5">
-        <v>0</v>
-      </c>
-      <c r="I10" s="5">
-        <v>0</v>
-      </c>
-      <c r="J10" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="B11" s="10" t="s">
+      <c r="C13" s="5">
+        <v>15</v>
+      </c>
+      <c r="D13" s="5">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5">
+        <v>0</v>
+      </c>
+      <c r="F13" s="5">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5">
+        <v>0</v>
+      </c>
+      <c r="I13" s="5">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="5">
-        <v>15</v>
-      </c>
-      <c r="D11" s="5">
-        <v>0</v>
-      </c>
-      <c r="E11" s="5">
-        <v>0</v>
-      </c>
-      <c r="F11" s="5">
-        <v>0</v>
-      </c>
-      <c r="G11" s="5">
-        <v>0</v>
-      </c>
-      <c r="H11" s="5">
-        <v>15</v>
-      </c>
-      <c r="I11" s="5">
-        <v>0</v>
-      </c>
-      <c r="J11" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="10" t="s">
+      <c r="C14" s="5">
+        <v>15</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5">
+        <v>0</v>
+      </c>
+      <c r="F14" s="5">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5">
+        <v>15</v>
+      </c>
+      <c r="I14" s="5">
+        <v>0</v>
+      </c>
+      <c r="J14" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C12" s="5">
-        <v>15</v>
-      </c>
-      <c r="D12" s="5">
-        <v>0</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0</v>
-      </c>
-      <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="5">
-        <v>15</v>
-      </c>
-      <c r="H12" s="5">
-        <v>0</v>
-      </c>
-      <c r="I12" s="5">
-        <v>0</v>
-      </c>
-      <c r="J12" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="B13" s="10" t="s">
+      <c r="C15" s="5">
+        <v>15</v>
+      </c>
+      <c r="D15" s="5">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0</v>
+      </c>
+      <c r="F15" s="5">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5">
+        <v>15</v>
+      </c>
+      <c r="H15" s="5">
+        <v>0</v>
+      </c>
+      <c r="I15" s="5">
+        <v>0</v>
+      </c>
+      <c r="J15" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="5">
-        <v>15</v>
-      </c>
-      <c r="D13" s="5">
-        <v>0</v>
-      </c>
-      <c r="E13" s="5">
-        <v>0</v>
-      </c>
-      <c r="F13" s="5">
-        <v>0</v>
-      </c>
-      <c r="G13" s="5">
-        <v>15</v>
-      </c>
-      <c r="H13" s="5">
-        <v>0</v>
-      </c>
-      <c r="I13" s="5">
-        <v>0</v>
-      </c>
-      <c r="J13" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="B14" s="10" t="s">
+      <c r="C16" s="5">
+        <v>15</v>
+      </c>
+      <c r="D16" s="5">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5">
+        <v>0</v>
+      </c>
+      <c r="F16" s="5">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5">
+        <v>15</v>
+      </c>
+      <c r="H16" s="5">
+        <v>0</v>
+      </c>
+      <c r="I16" s="5">
+        <v>0</v>
+      </c>
+      <c r="J16" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="5">
-        <v>15</v>
-      </c>
-      <c r="D14" s="5">
-        <v>0</v>
-      </c>
-      <c r="E14" s="5">
-        <v>0</v>
-      </c>
-      <c r="F14" s="5">
-        <v>0</v>
-      </c>
-      <c r="G14" s="5">
-        <v>0</v>
-      </c>
-      <c r="H14" s="5">
-        <v>0</v>
-      </c>
-      <c r="I14" s="5">
-        <v>0</v>
-      </c>
-      <c r="J14" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="B15" s="10" t="s">
+      <c r="C17" s="5">
+        <v>15</v>
+      </c>
+      <c r="D17" s="5">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5">
+        <v>0</v>
+      </c>
+      <c r="F17" s="5">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5">
+        <v>0</v>
+      </c>
+      <c r="I17" s="5">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C15" s="5">
-        <v>15</v>
-      </c>
-      <c r="D15" s="5">
-        <v>0</v>
-      </c>
-      <c r="E15" s="5">
-        <v>0</v>
-      </c>
-      <c r="F15" s="5">
-        <v>0</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0</v>
-      </c>
-      <c r="H15" s="5">
-        <v>15</v>
-      </c>
-      <c r="I15" s="5">
-        <v>0</v>
-      </c>
-      <c r="J15" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="B16" s="10" t="s">
+      <c r="C18" s="5">
+        <v>15</v>
+      </c>
+      <c r="D18" s="5">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5">
+        <v>0</v>
+      </c>
+      <c r="F18" s="5">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5">
+        <v>15</v>
+      </c>
+      <c r="I18" s="5">
+        <v>0</v>
+      </c>
+      <c r="J18" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="B19" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C16" s="5">
-        <v>15</v>
-      </c>
-      <c r="D16" s="5">
-        <v>0</v>
-      </c>
-      <c r="E16" s="5">
-        <v>0</v>
-      </c>
-      <c r="F16" s="5">
-        <v>0</v>
-      </c>
-      <c r="G16" s="5">
-        <v>15</v>
-      </c>
-      <c r="H16" s="5">
-        <v>0</v>
-      </c>
-      <c r="I16" s="5">
-        <v>0</v>
-      </c>
-      <c r="J16" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="B17" s="10" t="s">
+      <c r="C19" s="5">
+        <v>15</v>
+      </c>
+      <c r="D19" s="5">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5">
+        <v>15</v>
+      </c>
+      <c r="H19" s="5">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5">
+        <v>0</v>
+      </c>
+      <c r="J19" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="5">
-        <v>15</v>
-      </c>
-      <c r="D17" s="5">
-        <v>0</v>
-      </c>
-      <c r="E17" s="5">
-        <v>0</v>
-      </c>
-      <c r="F17" s="5">
-        <v>0</v>
-      </c>
-      <c r="G17" s="5">
-        <v>15</v>
-      </c>
-      <c r="H17" s="5">
-        <v>0</v>
-      </c>
-      <c r="I17" s="5">
-        <v>0</v>
-      </c>
-      <c r="J17" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="B18" s="10" t="s">
+      <c r="C20" s="5">
+        <v>15</v>
+      </c>
+      <c r="D20" s="5">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5">
+        <v>0</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5">
+        <v>15</v>
+      </c>
+      <c r="H20" s="5">
+        <v>0</v>
+      </c>
+      <c r="I20" s="5">
+        <v>0</v>
+      </c>
+      <c r="J20" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="B21" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="5">
-        <v>15</v>
-      </c>
-      <c r="D18" s="5">
-        <v>0</v>
-      </c>
-      <c r="E18" s="5">
-        <v>0</v>
-      </c>
-      <c r="F18" s="5">
-        <v>0</v>
-      </c>
-      <c r="G18" s="5">
-        <v>0</v>
-      </c>
-      <c r="H18" s="5">
-        <v>0</v>
-      </c>
-      <c r="I18" s="5">
-        <v>0</v>
-      </c>
-      <c r="J18" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="B19" s="10" t="s">
+      <c r="C21" s="5">
+        <v>15</v>
+      </c>
+      <c r="D21" s="5">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5">
+        <v>0</v>
+      </c>
+      <c r="I21" s="5">
+        <v>0</v>
+      </c>
+      <c r="J21" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="5">
-        <v>15</v>
-      </c>
-      <c r="D19" s="5">
-        <v>0</v>
-      </c>
-      <c r="E19" s="5">
-        <v>0</v>
-      </c>
-      <c r="F19" s="5">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5">
-        <v>15</v>
-      </c>
-      <c r="I19" s="5">
-        <v>0</v>
-      </c>
-      <c r="J19" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A20" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="B20" s="10" t="s">
+      <c r="C22" s="5">
+        <v>15</v>
+      </c>
+      <c r="D22" s="5">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5">
+        <v>15</v>
+      </c>
+      <c r="I22" s="5">
+        <v>0</v>
+      </c>
+      <c r="J22" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C20" s="5">
-        <v>15</v>
-      </c>
-      <c r="D20" s="5">
-        <v>0</v>
-      </c>
-      <c r="E20" s="5">
-        <v>0</v>
-      </c>
-      <c r="F20" s="5">
-        <v>0</v>
-      </c>
-      <c r="G20" s="5">
-        <v>15</v>
-      </c>
-      <c r="H20" s="5">
-        <v>0</v>
-      </c>
-      <c r="I20" s="5">
-        <v>0</v>
-      </c>
-      <c r="J20" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A21" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="B21" s="10" t="s">
+      <c r="C23" s="5">
+        <v>15</v>
+      </c>
+      <c r="D23" s="5">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0</v>
+      </c>
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5">
+        <v>15</v>
+      </c>
+      <c r="H23" s="5">
+        <v>0</v>
+      </c>
+      <c r="I23" s="5">
+        <v>0</v>
+      </c>
+      <c r="J23" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C21" s="5">
-        <v>15</v>
-      </c>
-      <c r="D21" s="5">
-        <v>0</v>
-      </c>
-      <c r="E21" s="5">
-        <v>0</v>
-      </c>
-      <c r="F21" s="5">
-        <v>0</v>
-      </c>
-      <c r="G21" s="5">
-        <v>15</v>
-      </c>
-      <c r="H21" s="5">
-        <v>0</v>
-      </c>
-      <c r="I21" s="5">
-        <v>0</v>
-      </c>
-      <c r="J21" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="C24" s="5">
+        <v>15</v>
+      </c>
+      <c r="D24" s="5">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5">
+        <v>0</v>
+      </c>
+      <c r="F24" s="5">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5">
+        <v>15</v>
+      </c>
+      <c r="H24" s="5">
+        <v>0</v>
+      </c>
+      <c r="I24" s="5">
+        <v>0</v>
+      </c>
+      <c r="J24" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="B25" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="5">
-        <v>15</v>
-      </c>
-      <c r="D22" s="5">
-        <v>0</v>
-      </c>
-      <c r="E22" s="5">
-        <v>0</v>
-      </c>
-      <c r="F22" s="5">
-        <v>0</v>
-      </c>
-      <c r="G22" s="5">
-        <v>0</v>
-      </c>
-      <c r="H22" s="5">
-        <v>0</v>
-      </c>
-      <c r="I22" s="5">
-        <v>0</v>
-      </c>
-      <c r="J22" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A23" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="B23" s="10" t="s">
+      <c r="C25" s="5">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5">
+        <v>0</v>
+      </c>
+      <c r="H25" s="5">
+        <v>0</v>
+      </c>
+      <c r="I25" s="5">
+        <v>0</v>
+      </c>
+      <c r="J25" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C23" s="5">
-        <v>15</v>
-      </c>
-      <c r="D23" s="5">
-        <v>0</v>
-      </c>
-      <c r="E23" s="5">
-        <v>0</v>
-      </c>
-      <c r="F23" s="5">
-        <v>0</v>
-      </c>
-      <c r="G23" s="5">
-        <v>0</v>
-      </c>
-      <c r="H23" s="5">
-        <v>15</v>
-      </c>
-      <c r="I23" s="5">
-        <v>0</v>
-      </c>
-      <c r="J23" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A24" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="C26" s="5">
+        <v>15</v>
+      </c>
+      <c r="D26" s="5">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5">
+        <v>15</v>
+      </c>
+      <c r="I26" s="5">
+        <v>0</v>
+      </c>
+      <c r="J26" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="B27" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C24" s="5">
-        <v>15</v>
-      </c>
-      <c r="D24" s="5">
-        <v>0</v>
-      </c>
-      <c r="E24" s="5">
-        <v>0</v>
-      </c>
-      <c r="F24" s="5">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5">
-        <v>15</v>
-      </c>
-      <c r="H24" s="5">
-        <v>0</v>
-      </c>
-      <c r="I24" s="5">
-        <v>0</v>
-      </c>
-      <c r="J24" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A25" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C25" s="5">
-        <v>15</v>
-      </c>
-      <c r="D25" s="5">
-        <v>0</v>
-      </c>
-      <c r="E25" s="5">
-        <v>0</v>
-      </c>
-      <c r="F25" s="5">
-        <v>0</v>
-      </c>
-      <c r="G25" s="5">
-        <v>15</v>
-      </c>
-      <c r="H25" s="5">
-        <v>0</v>
-      </c>
-      <c r="I25" s="5">
-        <v>0</v>
-      </c>
-      <c r="J25" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A26" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="B26" s="10" t="s">
+      <c r="C27" s="5">
+        <v>15</v>
+      </c>
+      <c r="D27" s="5">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5">
+        <v>15</v>
+      </c>
+      <c r="H27" s="5">
+        <v>0</v>
+      </c>
+      <c r="I27" s="5">
+        <v>0</v>
+      </c>
+      <c r="J27" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C26" s="5">
-        <v>15</v>
-      </c>
-      <c r="D26" s="5">
-        <v>0</v>
-      </c>
-      <c r="E26" s="5">
-        <v>0</v>
-      </c>
-      <c r="F26" s="5">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5">
-        <v>0</v>
-      </c>
-      <c r="H26" s="5">
-        <v>0</v>
-      </c>
-      <c r="I26" s="5">
-        <v>0</v>
-      </c>
-      <c r="J26" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A27" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="B27" s="10" t="s">
+      <c r="C28" s="5">
+        <v>15</v>
+      </c>
+      <c r="D28" s="5">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5">
+        <v>0</v>
+      </c>
+      <c r="F28" s="5">
+        <v>0</v>
+      </c>
+      <c r="G28" s="5">
+        <v>0</v>
+      </c>
+      <c r="H28" s="5">
+        <v>0</v>
+      </c>
+      <c r="I28" s="5">
+        <v>0</v>
+      </c>
+      <c r="J28" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="B29" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="5">
-        <v>15</v>
-      </c>
-      <c r="D27" s="5">
-        <v>0</v>
-      </c>
-      <c r="E27" s="5">
-        <v>0</v>
-      </c>
-      <c r="F27" s="5">
-        <v>0</v>
-      </c>
-      <c r="G27" s="5">
-        <v>0</v>
-      </c>
-      <c r="H27" s="5">
-        <v>15</v>
-      </c>
-      <c r="I27" s="5">
-        <v>0</v>
-      </c>
-      <c r="J27" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A28" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="B28" s="10" t="s">
+      <c r="C29" s="5">
+        <v>15</v>
+      </c>
+      <c r="D29" s="5">
+        <v>0</v>
+      </c>
+      <c r="E29" s="5">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5">
+        <v>0</v>
+      </c>
+      <c r="G29" s="5">
+        <v>0</v>
+      </c>
+      <c r="H29" s="5">
+        <v>15</v>
+      </c>
+      <c r="I29" s="5">
+        <v>0</v>
+      </c>
+      <c r="J29" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="B30" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C28" s="5">
-        <v>15</v>
-      </c>
-      <c r="D28" s="5">
-        <v>0</v>
-      </c>
-      <c r="E28" s="5">
-        <v>0</v>
-      </c>
-      <c r="F28" s="5">
-        <v>0</v>
-      </c>
-      <c r="G28" s="5">
-        <v>15</v>
-      </c>
-      <c r="H28" s="5">
-        <v>0</v>
-      </c>
-      <c r="I28" s="5">
-        <v>0</v>
-      </c>
-      <c r="J28" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A29" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="B29" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="5">
-        <v>15</v>
-      </c>
-      <c r="D29" s="5">
-        <v>0</v>
-      </c>
-      <c r="E29" s="5">
-        <v>0</v>
-      </c>
-      <c r="F29" s="5">
-        <v>0</v>
-      </c>
-      <c r="G29" s="5">
-        <v>15</v>
-      </c>
-      <c r="H29" s="5">
-        <v>0</v>
-      </c>
-      <c r="I29" s="5">
-        <v>0</v>
-      </c>
-      <c r="J29" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A30" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>11</v>
-      </c>
       <c r="C30" s="5">
         <v>15</v>
       </c>
@@ -11322,7 +11293,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="5">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H30" s="5">
         <v>0</v>
@@ -11336,811 +11307,811 @@
     </row>
     <row r="31" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B31" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="5">
+        <v>15</v>
+      </c>
+      <c r="D31" s="5">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5">
+        <v>0</v>
+      </c>
+      <c r="G31" s="5">
+        <v>15</v>
+      </c>
+      <c r="H31" s="5">
+        <v>0</v>
+      </c>
+      <c r="I31" s="5">
+        <v>0</v>
+      </c>
+      <c r="J31" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B32" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="5">
+        <v>15</v>
+      </c>
+      <c r="D32" s="5">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5">
+        <v>0</v>
+      </c>
+      <c r="I32" s="5">
+        <v>0</v>
+      </c>
+      <c r="J32" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="B33" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C31" s="5">
-        <v>15</v>
-      </c>
-      <c r="D31" s="5">
-        <v>0</v>
-      </c>
-      <c r="E31" s="5">
-        <v>0</v>
-      </c>
-      <c r="F31" s="5">
-        <v>0</v>
-      </c>
-      <c r="G31" s="5">
-        <v>0</v>
-      </c>
-      <c r="H31" s="5">
-        <v>15</v>
-      </c>
-      <c r="I31" s="5">
-        <v>0</v>
-      </c>
-      <c r="J31" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A32" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="B32" s="10" t="s">
+      <c r="C33" s="5">
+        <v>15</v>
+      </c>
+      <c r="D33" s="5">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5">
+        <v>0</v>
+      </c>
+      <c r="F33" s="5">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5">
+        <v>15</v>
+      </c>
+      <c r="I33" s="5">
+        <v>0</v>
+      </c>
+      <c r="J33" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B34" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C32" s="5">
-        <v>15</v>
-      </c>
-      <c r="D32" s="5">
-        <v>0</v>
-      </c>
-      <c r="E32" s="5">
-        <v>0</v>
-      </c>
-      <c r="F32" s="5">
-        <v>0</v>
-      </c>
-      <c r="G32" s="5">
-        <v>15</v>
-      </c>
-      <c r="H32" s="5">
-        <v>0</v>
-      </c>
-      <c r="I32" s="5">
-        <v>0</v>
-      </c>
-      <c r="J32" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A33" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="B33" s="10" t="s">
+      <c r="C34" s="5">
+        <v>15</v>
+      </c>
+      <c r="D34" s="5">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5">
+        <v>0</v>
+      </c>
+      <c r="F34" s="5">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5">
+        <v>15</v>
+      </c>
+      <c r="H34" s="5">
+        <v>0</v>
+      </c>
+      <c r="I34" s="5">
+        <v>0</v>
+      </c>
+      <c r="J34" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B35" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C35" s="5">
+        <v>15</v>
+      </c>
+      <c r="D35" s="5">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5">
+        <v>0</v>
+      </c>
+      <c r="F35" s="5">
+        <v>0</v>
+      </c>
+      <c r="G35" s="5">
+        <v>0</v>
+      </c>
+      <c r="H35" s="5">
+        <v>0</v>
+      </c>
+      <c r="I35" s="5">
+        <v>0</v>
+      </c>
+      <c r="J35" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="5">
+        <v>15</v>
+      </c>
+      <c r="D36" s="5">
+        <v>0</v>
+      </c>
+      <c r="E36" s="5">
+        <v>0</v>
+      </c>
+      <c r="F36" s="5">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5">
+        <v>0</v>
+      </c>
+      <c r="H36" s="5">
+        <v>15</v>
+      </c>
+      <c r="I36" s="5">
+        <v>0</v>
+      </c>
+      <c r="J36" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="5">
+        <v>15</v>
+      </c>
+      <c r="D37" s="5">
+        <v>0</v>
+      </c>
+      <c r="E37" s="5">
+        <v>0</v>
+      </c>
+      <c r="F37" s="5">
+        <v>0</v>
+      </c>
+      <c r="G37" s="5">
+        <v>15</v>
+      </c>
+      <c r="H37" s="5">
+        <v>0</v>
+      </c>
+      <c r="I37" s="5">
+        <v>0</v>
+      </c>
+      <c r="J37" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B38" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C33" s="5">
-        <v>15</v>
-      </c>
-      <c r="D33" s="5">
-        <v>0</v>
-      </c>
-      <c r="E33" s="5">
-        <v>0</v>
-      </c>
-      <c r="F33" s="5">
-        <v>0</v>
-      </c>
-      <c r="G33" s="5">
-        <v>15</v>
-      </c>
-      <c r="H33" s="5">
-        <v>0</v>
-      </c>
-      <c r="I33" s="5">
-        <v>0</v>
-      </c>
-      <c r="J33" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A34" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="B34" s="10" t="s">
+      <c r="C38" s="5">
+        <v>15</v>
+      </c>
+      <c r="D38" s="5">
+        <v>0</v>
+      </c>
+      <c r="E38" s="5">
+        <v>0</v>
+      </c>
+      <c r="F38" s="5">
+        <v>0</v>
+      </c>
+      <c r="G38" s="5">
+        <v>15</v>
+      </c>
+      <c r="H38" s="5">
+        <v>0</v>
+      </c>
+      <c r="I38" s="5">
+        <v>0</v>
+      </c>
+      <c r="J38" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="B39" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C34" s="5">
-        <v>15</v>
-      </c>
-      <c r="D34" s="5">
-        <v>0</v>
-      </c>
-      <c r="E34" s="5">
-        <v>0</v>
-      </c>
-      <c r="F34" s="5">
-        <v>0</v>
-      </c>
-      <c r="G34" s="5">
-        <v>0</v>
-      </c>
-      <c r="H34" s="5">
-        <v>0</v>
-      </c>
-      <c r="I34" s="5">
-        <v>0</v>
-      </c>
-      <c r="J34" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A35" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="B35" s="10" t="s">
+      <c r="C39" s="5">
+        <v>15</v>
+      </c>
+      <c r="D39" s="5">
+        <v>0</v>
+      </c>
+      <c r="E39" s="5">
+        <v>0</v>
+      </c>
+      <c r="F39" s="5">
+        <v>0</v>
+      </c>
+      <c r="G39" s="5">
+        <v>0</v>
+      </c>
+      <c r="H39" s="5">
+        <v>0</v>
+      </c>
+      <c r="I39" s="5">
+        <v>0</v>
+      </c>
+      <c r="J39" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="B40" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C35" s="5">
-        <v>15</v>
-      </c>
-      <c r="D35" s="5">
-        <v>0</v>
-      </c>
-      <c r="E35" s="5">
-        <v>0</v>
-      </c>
-      <c r="F35" s="5">
-        <v>0</v>
-      </c>
-      <c r="G35" s="5">
-        <v>0</v>
-      </c>
-      <c r="H35" s="5">
-        <v>15</v>
-      </c>
-      <c r="I35" s="5">
-        <v>0</v>
-      </c>
-      <c r="J35" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A36" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="B36" s="10" t="s">
+      <c r="C40" s="5">
+        <v>15</v>
+      </c>
+      <c r="D40" s="5">
+        <v>0</v>
+      </c>
+      <c r="E40" s="5">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5">
+        <v>0</v>
+      </c>
+      <c r="G40" s="5">
+        <v>0</v>
+      </c>
+      <c r="H40" s="5">
+        <v>15</v>
+      </c>
+      <c r="I40" s="5">
+        <v>0</v>
+      </c>
+      <c r="J40" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="B41" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="5">
-        <v>15</v>
-      </c>
-      <c r="D36" s="5">
-        <v>0</v>
-      </c>
-      <c r="E36" s="5">
-        <v>0</v>
-      </c>
-      <c r="F36" s="5">
-        <v>0</v>
-      </c>
-      <c r="G36" s="5">
-        <v>15</v>
-      </c>
-      <c r="H36" s="5">
-        <v>0</v>
-      </c>
-      <c r="I36" s="5">
-        <v>0</v>
-      </c>
-      <c r="J36" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A37" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="B37" s="10" t="s">
+      <c r="C41" s="5">
+        <v>15</v>
+      </c>
+      <c r="D41" s="5">
+        <v>0</v>
+      </c>
+      <c r="E41" s="5">
+        <v>0</v>
+      </c>
+      <c r="F41" s="5">
+        <v>0</v>
+      </c>
+      <c r="G41" s="5">
+        <v>15</v>
+      </c>
+      <c r="H41" s="5">
+        <v>0</v>
+      </c>
+      <c r="I41" s="5">
+        <v>0</v>
+      </c>
+      <c r="J41" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="B42" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="5">
-        <v>15</v>
-      </c>
-      <c r="D37" s="5">
-        <v>0</v>
-      </c>
-      <c r="E37" s="5">
-        <v>0</v>
-      </c>
-      <c r="F37" s="5">
-        <v>0</v>
-      </c>
-      <c r="G37" s="5">
-        <v>15</v>
-      </c>
-      <c r="H37" s="5">
-        <v>0</v>
-      </c>
-      <c r="I37" s="5">
-        <v>0</v>
-      </c>
-      <c r="J37" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A38" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B38" s="10" t="s">
+      <c r="C42" s="5">
+        <v>15</v>
+      </c>
+      <c r="D42" s="5">
+        <v>0</v>
+      </c>
+      <c r="E42" s="5">
+        <v>0</v>
+      </c>
+      <c r="F42" s="5">
+        <v>0</v>
+      </c>
+      <c r="G42" s="5">
+        <v>15</v>
+      </c>
+      <c r="H42" s="5">
+        <v>0</v>
+      </c>
+      <c r="I42" s="5">
+        <v>0</v>
+      </c>
+      <c r="J42" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B43" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C38" s="5">
-        <v>15</v>
-      </c>
-      <c r="D38" s="5">
-        <v>0</v>
-      </c>
-      <c r="E38" s="5">
-        <v>0</v>
-      </c>
-      <c r="F38" s="5">
-        <v>0</v>
-      </c>
-      <c r="G38" s="5">
-        <v>0</v>
-      </c>
-      <c r="H38" s="5">
-        <v>0</v>
-      </c>
-      <c r="I38" s="5">
-        <v>0</v>
-      </c>
-      <c r="J38" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A39" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="B39" s="10" t="s">
+      <c r="C43" s="5">
+        <v>15</v>
+      </c>
+      <c r="D43" s="5">
+        <v>0</v>
+      </c>
+      <c r="E43" s="5">
+        <v>0</v>
+      </c>
+      <c r="F43" s="5">
+        <v>0</v>
+      </c>
+      <c r="G43" s="5">
+        <v>0</v>
+      </c>
+      <c r="H43" s="5">
+        <v>0</v>
+      </c>
+      <c r="I43" s="5">
+        <v>0</v>
+      </c>
+      <c r="J43" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B44" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C39" s="5">
-        <v>15</v>
-      </c>
-      <c r="D39" s="5">
-        <v>0</v>
-      </c>
-      <c r="E39" s="5">
-        <v>0</v>
-      </c>
-      <c r="F39" s="5">
-        <v>0</v>
-      </c>
-      <c r="G39" s="5">
-        <v>0</v>
-      </c>
-      <c r="H39" s="5">
-        <v>15</v>
-      </c>
-      <c r="I39" s="5">
-        <v>0</v>
-      </c>
-      <c r="J39" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A40" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="B40" s="10" t="s">
+      <c r="C44" s="5">
+        <v>15</v>
+      </c>
+      <c r="D44" s="5">
+        <v>0</v>
+      </c>
+      <c r="E44" s="5">
+        <v>0</v>
+      </c>
+      <c r="F44" s="5">
+        <v>0</v>
+      </c>
+      <c r="G44" s="5">
+        <v>0</v>
+      </c>
+      <c r="H44" s="5">
+        <v>15</v>
+      </c>
+      <c r="I44" s="5">
+        <v>0</v>
+      </c>
+      <c r="J44" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="B45" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C40" s="5">
-        <v>15</v>
-      </c>
-      <c r="D40" s="5">
-        <v>0</v>
-      </c>
-      <c r="E40" s="5">
-        <v>0</v>
-      </c>
-      <c r="F40" s="5">
-        <v>0</v>
-      </c>
-      <c r="G40" s="5">
-        <v>15</v>
-      </c>
-      <c r="H40" s="5">
-        <v>0</v>
-      </c>
-      <c r="I40" s="5">
-        <v>0</v>
-      </c>
-      <c r="J40" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A41" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="B41" s="10" t="s">
+      <c r="C45" s="5">
+        <v>15</v>
+      </c>
+      <c r="D45" s="5">
+        <v>0</v>
+      </c>
+      <c r="E45" s="5">
+        <v>0</v>
+      </c>
+      <c r="F45" s="5">
+        <v>0</v>
+      </c>
+      <c r="G45" s="5">
+        <v>15</v>
+      </c>
+      <c r="H45" s="5">
+        <v>0</v>
+      </c>
+      <c r="I45" s="5">
+        <v>0</v>
+      </c>
+      <c r="J45" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="B46" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C41" s="5">
-        <v>15</v>
-      </c>
-      <c r="D41" s="5">
-        <v>0</v>
-      </c>
-      <c r="E41" s="5">
-        <v>0</v>
-      </c>
-      <c r="F41" s="5">
-        <v>0</v>
-      </c>
-      <c r="G41" s="5">
-        <v>15</v>
-      </c>
-      <c r="H41" s="5">
-        <v>0</v>
-      </c>
-      <c r="I41" s="5">
-        <v>0</v>
-      </c>
-      <c r="J41" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A42" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="B42" s="10" t="s">
+      <c r="C46" s="5">
+        <v>15</v>
+      </c>
+      <c r="D46" s="5">
+        <v>0</v>
+      </c>
+      <c r="E46" s="5">
+        <v>0</v>
+      </c>
+      <c r="F46" s="5">
+        <v>0</v>
+      </c>
+      <c r="G46" s="5">
+        <v>15</v>
+      </c>
+      <c r="H46" s="5">
+        <v>0</v>
+      </c>
+      <c r="I46" s="5">
+        <v>0</v>
+      </c>
+      <c r="J46" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="B47" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C42" s="5">
-        <v>15</v>
-      </c>
-      <c r="D42" s="5">
-        <v>0</v>
-      </c>
-      <c r="E42" s="5">
-        <v>0</v>
-      </c>
-      <c r="F42" s="5">
-        <v>0</v>
-      </c>
-      <c r="G42" s="5">
-        <v>0</v>
-      </c>
-      <c r="H42" s="5">
-        <v>0</v>
-      </c>
-      <c r="I42" s="5">
-        <v>0</v>
-      </c>
-      <c r="J42" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A43" s="14" t="s">
-        <v>184</v>
-      </c>
-      <c r="B43" s="10" t="s">
+      <c r="C47" s="5">
+        <v>15</v>
+      </c>
+      <c r="D47" s="5">
+        <v>0</v>
+      </c>
+      <c r="E47" s="5">
+        <v>0</v>
+      </c>
+      <c r="F47" s="5">
+        <v>0</v>
+      </c>
+      <c r="G47" s="5">
+        <v>0</v>
+      </c>
+      <c r="H47" s="5">
+        <v>0</v>
+      </c>
+      <c r="I47" s="5">
+        <v>0</v>
+      </c>
+      <c r="J47" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="B48" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C43" s="5">
-        <v>15</v>
-      </c>
-      <c r="D43" s="5">
-        <v>0</v>
-      </c>
-      <c r="E43" s="5">
-        <v>0</v>
-      </c>
-      <c r="F43" s="5">
-        <v>0</v>
-      </c>
-      <c r="G43" s="5">
-        <v>0</v>
-      </c>
-      <c r="H43" s="5">
-        <v>15</v>
-      </c>
-      <c r="I43" s="5">
-        <v>0</v>
-      </c>
-      <c r="J43" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A44" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="B44" s="10" t="s">
+      <c r="C48" s="5">
+        <v>15</v>
+      </c>
+      <c r="D48" s="5">
+        <v>0</v>
+      </c>
+      <c r="E48" s="5">
+        <v>0</v>
+      </c>
+      <c r="F48" s="5">
+        <v>0</v>
+      </c>
+      <c r="G48" s="5">
+        <v>0</v>
+      </c>
+      <c r="H48" s="5">
+        <v>15</v>
+      </c>
+      <c r="I48" s="5">
+        <v>0</v>
+      </c>
+      <c r="J48" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C44" s="5">
-        <v>15</v>
-      </c>
-      <c r="D44" s="5">
-        <v>0</v>
-      </c>
-      <c r="E44" s="5">
-        <v>0</v>
-      </c>
-      <c r="F44" s="5">
-        <v>0</v>
-      </c>
-      <c r="G44" s="5">
-        <v>15</v>
-      </c>
-      <c r="H44" s="5">
-        <v>0</v>
-      </c>
-      <c r="I44" s="5">
-        <v>0</v>
-      </c>
-      <c r="J44" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A45" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="B45" s="10" t="s">
+      <c r="C49" s="5">
+        <v>15</v>
+      </c>
+      <c r="D49" s="5">
+        <v>0</v>
+      </c>
+      <c r="E49" s="5">
+        <v>0</v>
+      </c>
+      <c r="F49" s="5">
+        <v>0</v>
+      </c>
+      <c r="G49" s="5">
+        <v>15</v>
+      </c>
+      <c r="H49" s="5">
+        <v>0</v>
+      </c>
+      <c r="I49" s="5">
+        <v>0</v>
+      </c>
+      <c r="J49" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="B50" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="5">
-        <v>15</v>
-      </c>
-      <c r="D45" s="5">
-        <v>0</v>
-      </c>
-      <c r="E45" s="5">
-        <v>0</v>
-      </c>
-      <c r="F45" s="5">
-        <v>0</v>
-      </c>
-      <c r="G45" s="5">
-        <v>15</v>
-      </c>
-      <c r="H45" s="5">
-        <v>0</v>
-      </c>
-      <c r="I45" s="5">
-        <v>0</v>
-      </c>
-      <c r="J45" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A46" s="14" t="s">
-        <v>187</v>
-      </c>
-      <c r="B46" s="10" t="s">
+      <c r="C50" s="5">
+        <v>15</v>
+      </c>
+      <c r="D50" s="5">
+        <v>0</v>
+      </c>
+      <c r="E50" s="5">
+        <v>0</v>
+      </c>
+      <c r="F50" s="5">
+        <v>0</v>
+      </c>
+      <c r="G50" s="5">
+        <v>15</v>
+      </c>
+      <c r="H50" s="5">
+        <v>0</v>
+      </c>
+      <c r="I50" s="5">
+        <v>0</v>
+      </c>
+      <c r="J50" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B51" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C46" s="5">
-        <v>15</v>
-      </c>
-      <c r="D46" s="5">
-        <v>0</v>
-      </c>
-      <c r="E46" s="5">
-        <v>0</v>
-      </c>
-      <c r="F46" s="5">
-        <v>0</v>
-      </c>
-      <c r="G46" s="5">
-        <v>0</v>
-      </c>
-      <c r="H46" s="5">
-        <v>0</v>
-      </c>
-      <c r="I46" s="5">
-        <v>0</v>
-      </c>
-      <c r="J46" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A47" s="14" t="s">
-        <v>188</v>
-      </c>
-      <c r="B47" s="10" t="s">
+      <c r="C51" s="5">
+        <v>15</v>
+      </c>
+      <c r="D51" s="5">
+        <v>0</v>
+      </c>
+      <c r="E51" s="5">
+        <v>0</v>
+      </c>
+      <c r="F51" s="5">
+        <v>0</v>
+      </c>
+      <c r="G51" s="5">
+        <v>0</v>
+      </c>
+      <c r="H51" s="5">
+        <v>0</v>
+      </c>
+      <c r="I51" s="5">
+        <v>0</v>
+      </c>
+      <c r="J51" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="B52" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="C47" s="5">
-        <v>15</v>
-      </c>
-      <c r="D47" s="5">
-        <v>0</v>
-      </c>
-      <c r="E47" s="5">
-        <v>0</v>
-      </c>
-      <c r="F47" s="5">
-        <v>0</v>
-      </c>
-      <c r="G47" s="5">
-        <v>0</v>
-      </c>
-      <c r="H47" s="5">
-        <v>15</v>
-      </c>
-      <c r="I47" s="5">
-        <v>0</v>
-      </c>
-      <c r="J47" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A48" s="14" t="s">
-        <v>189</v>
-      </c>
-      <c r="B48" s="10" t="s">
+      <c r="C52" s="5">
+        <v>15</v>
+      </c>
+      <c r="D52" s="5">
+        <v>0</v>
+      </c>
+      <c r="E52" s="5">
+        <v>0</v>
+      </c>
+      <c r="F52" s="5">
+        <v>0</v>
+      </c>
+      <c r="G52" s="5">
+        <v>0</v>
+      </c>
+      <c r="H52" s="5">
+        <v>15</v>
+      </c>
+      <c r="I52" s="5">
+        <v>0</v>
+      </c>
+      <c r="J52" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="B53" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="C48" s="5">
-        <v>15</v>
-      </c>
-      <c r="D48" s="5">
-        <v>0</v>
-      </c>
-      <c r="E48" s="5">
-        <v>0</v>
-      </c>
-      <c r="F48" s="5">
-        <v>0</v>
-      </c>
-      <c r="G48" s="5">
-        <v>15</v>
-      </c>
-      <c r="H48" s="5">
-        <v>0</v>
-      </c>
-      <c r="I48" s="5">
-        <v>0</v>
-      </c>
-      <c r="J48" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A49" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="B49" s="10" t="s">
+      <c r="C53" s="5">
+        <v>15</v>
+      </c>
+      <c r="D53" s="5">
+        <v>0</v>
+      </c>
+      <c r="E53" s="5">
+        <v>0</v>
+      </c>
+      <c r="F53" s="5">
+        <v>0</v>
+      </c>
+      <c r="G53" s="5">
+        <v>15</v>
+      </c>
+      <c r="H53" s="5">
+        <v>0</v>
+      </c>
+      <c r="I53" s="5">
+        <v>0</v>
+      </c>
+      <c r="J53" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="B54" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="C49" s="5">
-        <v>15</v>
-      </c>
-      <c r="D49" s="5">
-        <v>0</v>
-      </c>
-      <c r="E49" s="5">
-        <v>0</v>
-      </c>
-      <c r="F49" s="5">
-        <v>0</v>
-      </c>
-      <c r="G49" s="5">
-        <v>15</v>
-      </c>
-      <c r="H49" s="5">
-        <v>0</v>
-      </c>
-      <c r="I49" s="5">
-        <v>0</v>
-      </c>
-      <c r="J49" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A50" s="14" t="s">
-        <v>191</v>
-      </c>
-      <c r="B50" s="10" t="s">
+      <c r="C54" s="5">
+        <v>15</v>
+      </c>
+      <c r="D54" s="5">
+        <v>0</v>
+      </c>
+      <c r="E54" s="5">
+        <v>0</v>
+      </c>
+      <c r="F54" s="5">
+        <v>0</v>
+      </c>
+      <c r="G54" s="5">
+        <v>15</v>
+      </c>
+      <c r="H54" s="5">
+        <v>0</v>
+      </c>
+      <c r="I54" s="5">
+        <v>0</v>
+      </c>
+      <c r="J54" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="B55" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="5">
+        <v>15</v>
+      </c>
+      <c r="D55" s="5">
+        <v>0</v>
+      </c>
+      <c r="E55" s="5">
+        <v>0</v>
+      </c>
+      <c r="F55" s="5">
+        <v>0</v>
+      </c>
+      <c r="G55" s="5">
+        <v>15</v>
+      </c>
+      <c r="H55" s="5">
+        <v>0</v>
+      </c>
+      <c r="I55" s="5">
+        <v>0</v>
+      </c>
+      <c r="J55" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="B56" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="C50" s="5">
-        <v>15</v>
-      </c>
-      <c r="D50" s="5">
-        <v>0</v>
-      </c>
-      <c r="E50" s="5">
-        <v>0</v>
-      </c>
-      <c r="F50" s="5">
-        <v>0</v>
-      </c>
-      <c r="G50" s="5">
-        <v>0</v>
-      </c>
-      <c r="H50" s="5">
-        <v>0</v>
-      </c>
-      <c r="I50" s="5">
-        <v>0</v>
-      </c>
-      <c r="J50" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A51" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="B51" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C51" s="5">
-        <v>15</v>
-      </c>
-      <c r="D51" s="5">
-        <v>0</v>
-      </c>
-      <c r="E51" s="5">
-        <v>0</v>
-      </c>
-      <c r="F51" s="5">
-        <v>0</v>
-      </c>
-      <c r="G51" s="5">
-        <v>0</v>
-      </c>
-      <c r="H51" s="5">
-        <v>15</v>
-      </c>
-      <c r="I51" s="5">
-        <v>0</v>
-      </c>
-      <c r="J51" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A52" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="B52" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C52" s="5">
-        <v>15</v>
-      </c>
-      <c r="D52" s="5">
-        <v>0</v>
-      </c>
-      <c r="E52" s="5">
-        <v>0</v>
-      </c>
-      <c r="F52" s="5">
-        <v>0</v>
-      </c>
-      <c r="G52" s="5">
-        <v>15</v>
-      </c>
-      <c r="H52" s="5">
-        <v>0</v>
-      </c>
-      <c r="I52" s="5">
-        <v>0</v>
-      </c>
-      <c r="J52" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A53" s="14" t="s">
-        <v>194</v>
-      </c>
-      <c r="B53" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C53" s="5">
-        <v>15</v>
-      </c>
-      <c r="D53" s="5">
-        <v>0</v>
-      </c>
-      <c r="E53" s="5">
-        <v>0</v>
-      </c>
-      <c r="F53" s="5">
-        <v>0</v>
-      </c>
-      <c r="G53" s="5">
-        <v>15</v>
-      </c>
-      <c r="H53" s="5">
-        <v>0</v>
-      </c>
-      <c r="I53" s="5">
-        <v>0</v>
-      </c>
-      <c r="J53" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A54" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="B54" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C54" s="5">
-        <v>15</v>
-      </c>
-      <c r="D54" s="5">
-        <v>0</v>
-      </c>
-      <c r="E54" s="5">
-        <v>0</v>
-      </c>
-      <c r="F54" s="5">
-        <v>0</v>
-      </c>
-      <c r="G54" s="5">
-        <v>0</v>
-      </c>
-      <c r="H54" s="5">
-        <v>0</v>
-      </c>
-      <c r="I54" s="5">
-        <v>0</v>
-      </c>
-      <c r="J54" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A55" s="14" t="s">
-        <v>196</v>
-      </c>
-      <c r="B55" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C55" s="5">
-        <v>15</v>
-      </c>
-      <c r="D55" s="5">
-        <v>0</v>
-      </c>
-      <c r="E55" s="5">
-        <v>0</v>
-      </c>
-      <c r="F55" s="5">
-        <v>0</v>
-      </c>
-      <c r="G55" s="5">
-        <v>0</v>
-      </c>
-      <c r="H55" s="5">
-        <v>15</v>
-      </c>
-      <c r="I55" s="5">
-        <v>0</v>
-      </c>
-      <c r="J55" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A56" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="B56" s="10" t="s">
-        <v>72</v>
-      </c>
       <c r="C56" s="5">
         <v>15</v>
       </c>
@@ -12154,7 +12125,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="5">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H56" s="5">
         <v>0</v>
@@ -12166,9 +12137,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="14" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B57" s="10" t="s">
         <v>59</v>
@@ -12198,9 +12169,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B58" s="10" t="s">
         <v>72</v>
@@ -12230,9 +12201,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B59" s="10" t="s">
         <v>11</v>
@@ -12262,9 +12233,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B60" s="10" t="s">
         <v>59</v>
@@ -12294,9 +12265,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B61" s="10" t="s">
         <v>72</v>
@@ -12326,9 +12297,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B62" s="10" t="s">
         <v>11</v>
@@ -12358,9 +12329,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="14" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B63" s="10" t="s">
         <v>59</v>
@@ -12390,9 +12361,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="14" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B64" s="10" t="s">
         <v>72</v>
@@ -12422,9 +12393,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="14" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B65" s="10" t="s">
         <v>11</v>
@@ -12454,9 +12425,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="14" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B66" s="10" t="s">
         <v>59</v>
@@ -12486,9 +12457,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="14" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B67" s="10" t="s">
         <v>72</v>
@@ -12518,9 +12489,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="14" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>11</v>
@@ -12550,9 +12521,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="14" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B69" s="10" t="s">
         <v>59</v>
@@ -12582,9 +12553,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="14" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B70" s="10" t="s">
         <v>72</v>
@@ -12614,9 +12585,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="14" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B71" s="10" t="s">
         <v>11</v>
@@ -12646,9 +12617,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="14" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B72" s="10" t="s">
         <v>59</v>
@@ -12678,104 +12649,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A73" s="14" t="s">
-        <v>214</v>
-      </c>
-      <c r="B73" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C73" s="5">
-        <v>15</v>
-      </c>
-      <c r="D73" s="5">
-        <v>0</v>
-      </c>
-      <c r="E73" s="5">
-        <v>0</v>
-      </c>
-      <c r="F73" s="5">
-        <v>0</v>
-      </c>
-      <c r="G73" s="5">
-        <v>15</v>
-      </c>
-      <c r="H73" s="5">
-        <v>0</v>
-      </c>
-      <c r="I73" s="5">
-        <v>0</v>
-      </c>
-      <c r="J73" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A74" s="14" t="s">
-        <v>215</v>
-      </c>
-      <c r="B74" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="C74" s="5">
-        <v>15</v>
-      </c>
-      <c r="D74" s="5">
-        <v>0</v>
-      </c>
-      <c r="E74" s="5">
-        <v>0</v>
-      </c>
-      <c r="F74" s="5">
-        <v>0</v>
-      </c>
-      <c r="G74" s="5">
-        <v>0</v>
-      </c>
-      <c r="H74" s="5">
-        <v>0</v>
-      </c>
-      <c r="I74" s="5">
-        <v>0</v>
-      </c>
-      <c r="J74" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" ht="16" x14ac:dyDescent="0.2">
-      <c r="A75" s="14" t="s">
-        <v>216</v>
-      </c>
-      <c r="B75" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C75" s="5">
-        <v>15</v>
-      </c>
-      <c r="D75" s="5">
-        <v>0</v>
-      </c>
-      <c r="E75" s="5">
-        <v>0</v>
-      </c>
-      <c r="F75" s="5">
-        <v>0</v>
-      </c>
-      <c r="G75" s="5">
-        <v>15</v>
-      </c>
-      <c r="H75" s="5">
-        <v>0</v>
-      </c>
-      <c r="I75" s="5">
-        <v>0</v>
-      </c>
-      <c r="J75" s="9">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I75" xr:uid="{B237460F-1A26-43E8-9FBD-2B515F45BBA9}"/>
+  <autoFilter ref="A1:I72" xr:uid="{B237460F-1A26-43E8-9FBD-2B515F45BBA9}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="sw10018sf"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
added request body logging for endpoints, that get called with a request body
</commit_message>
<xml_diff>
--- a/packages/backend/files/Produktionszeit_Warenfluss_Hackathon_Teilnehmer.xlsx
+++ b/packages/backend/files/Produktionszeit_Warenfluss_Hackathon_Teilnehmer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ap8c3/IdeaProjects/Hackathon/eleo-mind/packages/backend/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13D3DB1-55DE-B34A-B882-2ABBE7A9C9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C052F07-A7AE-A249-9EB5-FFD35E62D8B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="17380" activeTab="4" xr2:uid="{89DEC141-2149-4C1E-98A2-7345C7C4F172}"/>
   </bookViews>
@@ -10328,7 +10328,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B237460F-1A26-43E8-9FBD-2B515F45BBA9}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:J72"/>
@@ -10377,7 +10377,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>146</v>
       </c>
@@ -10409,7 +10409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>147</v>
       </c>
@@ -10441,7 +10441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>148</v>
       </c>
@@ -10473,7 +10473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
         <v>149</v>
       </c>
@@ -10505,7 +10505,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>150</v>
       </c>
@@ -10537,7 +10537,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
         <v>151</v>
       </c>
@@ -10569,7 +10569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
         <v>152</v>
       </c>
@@ -10601,7 +10601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
         <v>153</v>
       </c>
@@ -10633,7 +10633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
         <v>154</v>
       </c>
@@ -10665,7 +10665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
         <v>155</v>
       </c>
@@ -10697,7 +10697,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>156</v>
       </c>
@@ -10729,7 +10729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
         <v>157</v>
       </c>
@@ -10761,7 +10761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
         <v>158</v>
       </c>
@@ -10793,7 +10793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
         <v>159</v>
       </c>
@@ -10825,7 +10825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
         <v>160</v>
       </c>
@@ -10857,7 +10857,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
         <v>161</v>
       </c>
@@ -10889,7 +10889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
         <v>162</v>
       </c>
@@ -10921,7 +10921,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
         <v>163</v>
       </c>
@@ -10953,7 +10953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
         <v>164</v>
       </c>
@@ -10985,7 +10985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
         <v>165</v>
       </c>
@@ -11017,7 +11017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
         <v>166</v>
       </c>
@@ -11049,7 +11049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
         <v>167</v>
       </c>
@@ -11081,7 +11081,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
         <v>168</v>
       </c>
@@ -11113,7 +11113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="14" t="s">
         <v>169</v>
       </c>
@@ -11145,7 +11145,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
         <v>170</v>
       </c>
@@ -11177,7 +11177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="14" t="s">
         <v>171</v>
       </c>
@@ -11209,7 +11209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
         <v>172</v>
       </c>
@@ -11241,7 +11241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="14" t="s">
         <v>173</v>
       </c>
@@ -11273,7 +11273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
         <v>174</v>
       </c>
@@ -11337,7 +11337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
         <v>176</v>
       </c>
@@ -11369,7 +11369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="14" t="s">
         <v>177</v>
       </c>
@@ -11401,7 +11401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="14" t="s">
         <v>178</v>
       </c>
@@ -11433,7 +11433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
         <v>179</v>
       </c>
@@ -11465,7 +11465,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
         <v>180</v>
       </c>
@@ -11497,7 +11497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
         <v>181</v>
       </c>
@@ -11529,7 +11529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A38" s="14" t="s">
         <v>182</v>
       </c>
@@ -11561,7 +11561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
         <v>183</v>
       </c>
@@ -11593,7 +11593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
         <v>184</v>
       </c>
@@ -11625,7 +11625,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
         <v>185</v>
       </c>
@@ -11657,7 +11657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
         <v>186</v>
       </c>
@@ -11689,7 +11689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A43" s="14" t="s">
         <v>187</v>
       </c>
@@ -11721,7 +11721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A44" s="14" t="s">
         <v>188</v>
       </c>
@@ -11753,7 +11753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A45" s="14" t="s">
         <v>189</v>
       </c>
@@ -11785,7 +11785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
         <v>190</v>
       </c>
@@ -11817,7 +11817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="14" t="s">
         <v>191</v>
       </c>
@@ -11849,7 +11849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
         <v>192</v>
       </c>
@@ -11881,7 +11881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A49" s="14" t="s">
         <v>193</v>
       </c>
@@ -11913,7 +11913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
         <v>194</v>
       </c>
@@ -11945,7 +11945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A51" s="14" t="s">
         <v>195</v>
       </c>
@@ -11977,7 +11977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
         <v>196</v>
       </c>
@@ -12009,7 +12009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A53" s="14" t="s">
         <v>197</v>
       </c>
@@ -12041,7 +12041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
         <v>198</v>
       </c>
@@ -12073,7 +12073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A55" s="14" t="s">
         <v>199</v>
       </c>
@@ -12105,7 +12105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
         <v>200</v>
       </c>
@@ -12137,7 +12137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A57" s="14" t="s">
         <v>201</v>
       </c>
@@ -12169,7 +12169,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
         <v>202</v>
       </c>
@@ -12201,7 +12201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
         <v>203</v>
       </c>
@@ -12233,7 +12233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>204</v>
       </c>
@@ -12265,7 +12265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
         <v>205</v>
       </c>
@@ -12297,7 +12297,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
         <v>206</v>
       </c>
@@ -12329,7 +12329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A63" s="14" t="s">
         <v>207</v>
       </c>
@@ -12361,7 +12361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A64" s="14" t="s">
         <v>208</v>
       </c>
@@ -12393,7 +12393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A65" s="14" t="s">
         <v>209</v>
       </c>
@@ -12425,7 +12425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A66" s="14" t="s">
         <v>210</v>
       </c>
@@ -12457,7 +12457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A67" s="14" t="s">
         <v>211</v>
       </c>
@@ -12489,7 +12489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A68" s="14" t="s">
         <v>212</v>
       </c>
@@ -12521,7 +12521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A69" s="14" t="s">
         <v>213</v>
       </c>
@@ -12553,7 +12553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A70" s="14" t="s">
         <v>214</v>
       </c>
@@ -12585,7 +12585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A71" s="14" t="s">
         <v>215</v>
       </c>
@@ -12617,7 +12617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="16" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" ht="16" x14ac:dyDescent="0.2">
       <c r="A72" s="14" t="s">
         <v>216</v>
       </c>
@@ -12650,13 +12650,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I72" xr:uid="{B237460F-1A26-43E8-9FBD-2B515F45BBA9}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="sw10018sf"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I72" xr:uid="{B237460F-1A26-43E8-9FBD-2B515F45BBA9}"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>